<commit_message>
style: normalize formatting and trailing newlines across test suites and QA tools
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -3493,11 +3493,11 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22 11:57:03</t>
+          <t>2026-10-22 12:20:21</t>
         </is>
       </c>
       <c r="K48" s="4" t="n">
-        <v>0.1246</v>
+        <v>0.1829</v>
       </c>
       <c r="L48" s="3" t="inlineStr"/>
       <c r="M48" s="4" t="inlineStr">
@@ -3554,11 +3554,11 @@
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22 11:57:03</t>
+          <t>2026-10-22 12:20:21</t>
         </is>
       </c>
       <c r="K49" s="4" t="n">
-        <v>0.2065</v>
+        <v>0.185</v>
       </c>
       <c r="L49" s="3" t="inlineStr"/>
       <c r="M49" s="4" t="inlineStr">
@@ -3615,11 +3615,11 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22 11:57:03</t>
+          <t>2026-10-22 12:20:21</t>
         </is>
       </c>
       <c r="K50" s="4" t="n">
-        <v>0.231</v>
+        <v>0.2811</v>
       </c>
       <c r="L50" s="3" t="inlineStr"/>
       <c r="M50" s="4" t="inlineStr">
@@ -3676,11 +3676,11 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22 11:57:04</t>
+          <t>2026-10-22 12:20:22</t>
         </is>
       </c>
       <c r="K51" s="4" t="n">
-        <v>0.3514</v>
+        <v>0.2727</v>
       </c>
       <c r="L51" s="3" t="inlineStr"/>
       <c r="M51" s="4" t="inlineStr">
@@ -3737,11 +3737,11 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22 11:57:04</t>
+          <t>2026-10-22 12:20:22</t>
         </is>
       </c>
       <c r="K52" s="4" t="n">
-        <v>0.0762</v>
+        <v>0.0585</v>
       </c>
       <c r="L52" s="3" t="inlineStr"/>
       <c r="M52" s="4" t="inlineStr">
@@ -3798,11 +3798,11 @@
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22 11:57:04</t>
+          <t>2026-10-22 12:20:22</t>
         </is>
       </c>
       <c r="K53" s="4" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="L53" s="3" t="inlineStr"/>
       <c r="M53" s="4" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4276,6 +4276,88 @@
       </c>
       <c r="I7" s="4" t="n">
         <v>44.88</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Run Timestamp</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Total Tests</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pass Rate (%)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Git Hash</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Duration (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-22 12:20:22</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>49c97f1</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>3.38</v>
       </c>
     </row>
   </sheetData>
@@ -5078,8 +5160,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>